<commit_message>
Add PCIE TestPlan Excel generated from GitHub tests
</commit_message>
<xml_diff>
--- a/Test_Output/PCIE/PCIE_TestPlan.xlsx
+++ b/Test_Output/PCIE/PCIE_TestPlan.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="TestPlan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="PCIE_TestPlan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,24 +417,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="105" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="83" customWidth="1" min="9" max="9"/>
-    <col width="122" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="122" customWidth="1" min="12" max="12"/>
-    <col width="122" customWidth="1" min="13" max="13"/>
-    <col width="73" customWidth="1" min="14" max="14"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -444,67 +428,57 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>IP_NAME</t>
+          <t>SS / Module</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>SS / Module</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Test Case Name</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Test Case Name</t>
+          <t>Test Description</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Test Description</t>
+          <t>Speed</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>Mode</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Mode</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Test Steps / Procedure</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Test Steps / Procedure</t>
+          <t>Impacted Registers</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Impacted Registers</t>
+          <t>Validation / Acceptance Criteria</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Validation / Acceptance Criteria</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
           <t>Gap Analysis</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Source File Path</t>
         </is>
       </c>
     </row>
@@ -521,22 +495,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PCIE Config Registers</t>
+          <t>pcie_cfg_wr_rd_test</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>cfg_wr_rd</t>
+          <t>pcie_cfg_wr_rd_test</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>pcie_cfg_wr_rd_test</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Validate default reset values and masked read/write behavior for selected PCIe configuration registers.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -551,38 +525,22 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Uses read_mask_array, write_mask_array, and skip_array to control RO/RW behavior.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>1. Read each address in addr_array and compare to default_value_array using read_mask_array.
-2. For each test pattern (0xAAAAAAAA, 0x55555555, 0xFFFFFFFF, 0x00000000), write to writable addresses (per write_mask_array).
-3. Read back each addressed register and compute expected using (data_wr &amp; write_mask_array) | (~write_mask_array &amp; default_value_array).
-4. Increment failure counters and log CFG_RST_FAIL/CFG_WR_FAIL on mismatches.
-5. Call finish(0) if no failures; otherwise call finish(1).</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>VENDOR_DEVICE_ID, STATUS_COMMAND, CLASSCODE, BAR0, INT_PIN</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Pass if def_fail_cnt == 0 and wr_fail_cnt == 0; no logs containing "CFG_RST_FAIL" or "CFG_WR_FAIL"; finish(0) is called.</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>- Default values are hardcoded to 0; true reset defaults are not validated.
-- No error handling around read_reg/write_reg operations.
-- Limited pattern coverage; no random or walking patterns.</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>TestRepo/pcie/pcie_cfg_wr_rd_test/pcie_cfg_wr_rd_test.c</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -599,22 +557,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PCIE DBI DSP Registers</t>
+          <t>pcie_dbi_dsp_reg_wr_rd_test</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>dbi_dsp_reg_wr_rd</t>
+          <t>pcie_dbi_dsp_reg_wr_rd_test</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>pcie_dbi_dsp_reg_wr_rd_test</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Verify default values and basic read/write for DBI DSP registers.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -629,37 +587,22 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Writes to all addresses without RO masking; skip_array not used.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>1. Read each DSP register and compare to default_value_array.
-2. For each pattern (0xAAAAAAAA, 0x55555555, 0x00000000), write the value to all registers.
-3. Read back each register and compare to the last written pattern.
-4. Increment def_fail_cnt or wr_fail_cnt and log DSP_RST_FAIL/DSP_WR_FAIL on mismatches.
-5. Call finish(0) if no failures; otherwise call finish(1).</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>CMD_STATUS, CFG_SETUP, OB_SIZE, IRQ_EOI</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Pass if def_fail_cnt == 0 and wr_fail_cnt == 0; no logs containing "DSP_RST_FAIL" or "DSP_WR_FAIL"; finish(0) is called.</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>- No read/write masks or RO handling; potential false failures on RO fields.
-- Default values hardcoded to 0; true reset defaults not validated.</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>TestRepo/pcie/pcie_dbi_dsp_reg_wr_rd_test/pcie_dbi_dsp_reg_wr_rd_test.c</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -676,22 +619,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PCIE DBI USP Registers</t>
+          <t>pcie_dbi_usp_reg_wr_rd_test</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>dbi_usp_reg_wr_rd</t>
+          <t>pcie_dbi_usp_reg_wr_rd_test</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>pcie_dbi_usp_reg_wr_rd_test</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Verify default values and read/write for DBI USP GPR registers.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -706,37 +649,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Single write pattern used; no RO masking.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>1. Read GPR registers and compare to default_value_array.
-2. Write 0xA5A5A5A5 to each GPR register.
-3. Read back each register and compare to 0xA5A5A5A5.
-4. Increment def_fail_cnt or wr_fail_cnt on mismatches.
-5. Call finish(0) if no failures; otherwise call finish(1).</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>GPR0, GPR1, GPR2</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Pass if def_fail_cnt == 0 and wr_fail_cnt == 0; finish(0) is called.</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>- No masking for RO or reserved bits; may not reflect true HW constraints.
-- Only one write pattern; limited data pattern coverage.</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>TestRepo/pcie/pcie_dbi_usp_reg_wr_rd_test/pcie_dbi_usp_reg_wr_rd_test.c</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -753,22 +681,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PCIE SII RC Registers</t>
+          <t>pcie_sii_rc_reg_wr_rd_test</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>sii_rc_reg_wr_rd</t>
+          <t>pcie_sii_rc_reg_wr_rd_test</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>pcie_sii_rc_reg_wr_rd_test</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Verify default values and read/write for SII Root Complex inbound address registers.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -783,37 +711,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Two write patterns; no RO masking.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>1. Read each SII RC register and compare to default_value_array.
-2. For each pattern (0xFFFFFFFF, 0x00000000), write the value to all registers.
-3. Read back each register and compare to the last written pattern.
-4. Increment def_fail_cnt or wr_fail_cnt on mismatches.
-5. Call finish(0) if no failures; otherwise call finish(1).</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>IB_BAR0, IB_START_LO, IB_OFFSET</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Pass if def_fail_cnt == 0 and wr_fail_cnt == 0; finish(0) is called.</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>- No handling for RO fields or field-level masks.
-- Limited pattern set; does not test address alignment or partial-width writes.</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>TestRepo/pcie/pcie_sii_rc_reg_wr_rd_test/pcie_sii_rc_reg_wr_rd_test.c</t>
+          <t>NA</t>
         </is>
       </c>
     </row>

</xml_diff>